<commit_message>
Restaurar estado de roles y logs web; integrar auditoria y matriz en documento Excel
</commit_message>
<xml_diff>
--- a/Matriz_de_Roles_y_Permisos_SGI.xlsx
+++ b/Matriz_de_Roles_y_Permisos_SGI.xlsx
@@ -4,11 +4,12 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView activeTab="1" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView activeTab="2" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
     <sheet name="Jerarquía de Roles" sheetId="1" r:id="rId4"/>
     <sheet name="Matriz Detallada" sheetId="2" r:id="rId5"/>
+    <sheet name="Logs y Auditoría" sheetId="3" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Matriz Detallada'!$A$4:$H$128</definedName>
@@ -18,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="361">
   <si>
     <t>SGI - SISTEMA DE GESTIÓN DE INVENTARIOS</t>
   </si>
@@ -519,6 +520,593 @@
   </si>
   <si>
     <t>Traslado - Ruta - modificar</t>
+  </si>
+  <si>
+    <t>SGI - SISTEMA DE GESTIÓN DE INVENTARIOS | GRUPO NODO</t>
+  </si>
+  <si>
+    <t>ESPECIFICACIÓN Y MATRIZ DE LOGS DE AUDITORÍA (ALTA, EDICIÓN, BAJA Y CONSUMO)</t>
+  </si>
+  <si>
+    <t>Control de trazabilidad de operaciones críticas: Creación, Modificación, Desincorporación y Salidas de Stock</t>
+  </si>
+  <si>
+    <t>RESUMEN EJECUTIVO DE EVENTOS DE AUDITORÍA</t>
+  </si>
+  <si>
+    <t>1. ALTA / CREACIÓN</t>
+  </si>
+  <si>
+    <t>Registro inicial de bienes fijos, consumibles, comerciales y vehículos.
+Captura: código, custodio, ubicación, fotos y factura.</t>
+  </si>
+  <si>
+    <t>2. EDICIÓN / CAMBIOS</t>
+  </si>
+  <si>
+    <t>Modificación de atributos, fotografías, números de serie o custodio.
+Captura: valores previos vs nuevos y justificación.</t>
+  </si>
+  <si>
+    <t>3. BAJA / DESCARTE</t>
+  </si>
+  <si>
+    <t>Desincorporación por daño irreparable, extravío u obsolescencia.
+Captura: motivo fundamentado y acta digital obligatoria.</t>
+  </si>
+  <si>
+    <t>4. CONSUMO DE STOCK</t>
+  </si>
+  <si>
+    <t>Disminución de existencias en consumibles con vale o motivo.
+Captura: cantidad consumida, solicitante y saldo en kardex.</t>
+  </si>
+  <si>
+    <t>5. REABASTECIMIENTO</t>
+  </si>
+  <si>
+    <t>Ingreso de compras y reposición de existencias de insumos.
+Captura: proveedor, remisión, unidades y saldo actualizado.</t>
+  </si>
+  <si>
+    <t>MATRIZ DETALLADA DE LOGS Y EVENTOS DE AUDITORÍA</t>
+  </si>
+  <si>
+    <t>ID Evento</t>
+  </si>
+  <si>
+    <t>Tipo de Acción</t>
+  </si>
+  <si>
+    <t>Módulo / Categoría</t>
+  </si>
+  <si>
+    <t>Disparador en Sistema (Trigger)</t>
+  </si>
+  <si>
+    <t>Campos Registrados (Tabla movimientos)</t>
+  </si>
+  <si>
+    <t>Impacto en Inventario / Kardex</t>
+  </si>
+  <si>
+    <t>Evidencia / Comprobante Requerido</t>
+  </si>
+  <si>
+    <t>Roles Autorizados</t>
+  </si>
+  <si>
+    <t>Ejemplo Descriptivo de Registro de Log</t>
+  </si>
+  <si>
+    <t>Criticidad</t>
+  </si>
+  <si>
+    <t>LOG-ACT-01</t>
+  </si>
+  <si>
+    <t>Creación / Alta</t>
+  </si>
+  <si>
+    <t>Activos Fijos</t>
+  </si>
+  <si>
+    <t>Al guardar nuevo producto en "Activos Fijos &gt; Crear"</t>
+  </si>
+  <si>
+    <t>id_producto, id_user, categoria='fijos', accion='Alta de producto', comentario, documentacion</t>
+  </si>
+  <si>
+    <t>Incrementa inventario activo; asigna número de inventario interno, ubicación física y custodio responsable.</t>
+  </si>
+  <si>
+    <t>Factura de adquisición, fotografía digital del activo y etiqueta de código de barras.</t>
+  </si>
+  <si>
+    <t>Super Admin, Administrador, Almacenistas</t>
+  </si>
+  <si>
+    <t>[Alta] Usuario 'juan.almacen' dio de alta Laptop Dell Latitude 5420 (INV-0042) en Depto TI.</t>
+  </si>
+  <si>
+    <t>Informativa</t>
+  </si>
+  <si>
+    <t>LOG-ACT-02</t>
+  </si>
+  <si>
+    <t>Edición / Modificación</t>
+  </si>
+  <si>
+    <t>Al presionar "Guardar Cambios" en ficha del activo fijo</t>
+  </si>
+  <si>
+    <t>id_producto, id_user, categoria='fijos', accion='Actualización de información', comentario con campos modificados</t>
+  </si>
+  <si>
+    <t>Actualiza ficha técnica, reasignación de ubicación o custodio; mantiene trazabilidad histórica.</t>
+  </si>
+  <si>
+    <t>Formato de resguardo interno firmado o evidencia fotográfica del estado actual.</t>
+  </si>
+  <si>
+    <t>Super Admin, Administrador</t>
+  </si>
+  <si>
+    <t>[Edición] Usuario 'admin@nodo.mx' cambió ubicación de Monitor LG de 'Piso 2' a 'Recepción'.</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>LOG-ACT-03</t>
+  </si>
+  <si>
+    <t>Baja / Descarte</t>
+  </si>
+  <si>
+    <t>Al seleccionar opción "Dar de Baja" o estado="baja" en formulario</t>
+  </si>
+  <si>
+    <t>id_producto, id_user, categoria='fijos', accion='Baja de producto', comentario (motivo), documentacion (acta)</t>
+  </si>
+  <si>
+    <t>Pasa a estatus 'baja' (inactivo); se excluye de listados operativos y se desvincula custodio.</t>
+  </si>
+  <si>
+    <t>Dictamen técnico de desecho, reporte de extravío o acta administrativa firmada.</t>
+  </si>
+  <si>
+    <t>[Baja] Usuario 'superadmin@nodo.mx' dio de baja Impresora HP LaserJet por falla de tarjeta madre irreparable.</t>
+  </si>
+  <si>
+    <t>Alta</t>
+  </si>
+  <si>
+    <t>LOG-CON-01</t>
+  </si>
+  <si>
+    <t>Consumibles</t>
+  </si>
+  <si>
+    <t>Al registrar nuevo consumible en catálogo de insumos</t>
+  </si>
+  <si>
+    <t>id_producto, id_user, categoria='consumibles', accion='Alta de consumible', comentario, foto</t>
+  </si>
+  <si>
+    <t>Crea ficha del insumo en catálogo; establece umbral de existencia mínima y alerta del 10%.</t>
+  </si>
+  <si>
+    <t>Ficha técnica del producto o comprobante de compra.</t>
+  </si>
+  <si>
+    <t>[Alta] Usuario 'pedro.almacen' registró insumo Tóner HP 85A Negro (Ubicación: Anaquel A-2).</t>
+  </si>
+  <si>
+    <t>LOG-CON-02</t>
+  </si>
+  <si>
+    <t>Consumo de Existencias</t>
+  </si>
+  <si>
+    <t>Al presionar "Ajustar Existencia &gt; Disminuir" en modal de consumibles</t>
+  </si>
+  <si>
+    <t>id_producto, id_user, categoria='consumibles', accion='Consumo', comentario (cantidad consumida y motivo)</t>
+  </si>
+  <si>
+    <t>Resta unidades al saldo actual. Si el saldo resultante es &lt;= 10%, detona alerta automática en el Dashboard.</t>
+  </si>
+  <si>
+    <t>Vale de entrega de insumos o registro de departamento/usuario solicitante.</t>
+  </si>
+  <si>
+    <t>Super Admin, Administrador, Almacenistas, Auxiliares</t>
+  </si>
+  <si>
+    <t>[Consumo] Usuario 'mario.aux' registró salida de 3 piezas de Tóner HP 85A para Área de Contabilidad. Saldo: 4.</t>
+  </si>
+  <si>
+    <t>LOG-CON-03</t>
+  </si>
+  <si>
+    <t>Reabastecimiento</t>
+  </si>
+  <si>
+    <t>Al presionar "Ajustar Existencia &gt; Aumentar" en modal de consumibles</t>
+  </si>
+  <si>
+    <t>id_producto, id_user, categoria='consumibles', accion='Reabastecimiento', comentario (unidades y remisión)</t>
+  </si>
+  <si>
+    <t>Suma unidades al saldo actual. Si el saldo supera el 10%, se desactiva la alerta de stock crítico.</t>
+  </si>
+  <si>
+    <t>Orden de compra, remisión del proveedor o factura de surtido.</t>
+  </si>
+  <si>
+    <t>[Reabastecimiento] Usuario 'pedro.almacen' ingresó 20 cajas de Hojas Carta. Saldo anterior: 3, Nuevo: 23.</t>
+  </si>
+  <si>
+    <t>LOG-CON-04</t>
+  </si>
+  <si>
+    <t>Baja / Ajuste Merma</t>
+  </si>
+  <si>
+    <t>Al ajustar saldo por daño, caducidad, merma o conteo físico</t>
+  </si>
+  <si>
+    <t>id_producto, id_user, categoria='consumibles', accion='Ajuste Merma', comentario justificativo</t>
+  </si>
+  <si>
+    <t>Ajusta la existencia física en kardex con motivo explícito de discrepancia o daño de material.</t>
+  </si>
+  <si>
+    <t>Acta de merma firmada por jefe de bodega y evidencia fotográfica del insumo dañado.</t>
+  </si>
+  <si>
+    <t>[Merma] Usuario 'admin@nodo.mx' dio de baja 4 litros de solvente por derrame en contenedor.</t>
+  </si>
+  <si>
+    <t>LOG-CPV-01</t>
+  </si>
+  <si>
+    <t>Compra-Venta</t>
+  </si>
+  <si>
+    <t>Al registrar artículo comercializable en catálogo compra/venta</t>
+  </si>
+  <si>
+    <t>id_producto, id_user, categoria='compraventa', accion='Alta producto comercial', comentario, precios</t>
+  </si>
+  <si>
+    <t>Ingresa producto con existencias vendibles, precio de costo y precio de lista al público.</t>
+  </si>
+  <si>
+    <t>Factura de compra del lote comercial y ficha de catálogo.</t>
+  </si>
+  <si>
+    <t>[Alta] Usuario 'carlos.almacen' ingresó 50 Rollos de Cable UTP Cat6 305m (Costo: $950, Venta: $1,450).</t>
+  </si>
+  <si>
+    <t>LOG-CPV-02</t>
+  </si>
+  <si>
+    <t>Edición / Precios</t>
+  </si>
+  <si>
+    <t>Al actualizar precios, márgenes o especificaciones del artículo</t>
+  </si>
+  <si>
+    <t>id_producto, id_user, categoria='compraventa', accion='Modificación de producto/precios', comentario</t>
+  </si>
+  <si>
+    <t>Actualiza los importes del sistema de cotización y venta en tiempo real.</t>
+  </si>
+  <si>
+    <t>Autorización de gerencia de operaciones o cambio de lista de precios de fabricante.</t>
+  </si>
+  <si>
+    <t>[Edición] Usuario 'admin@nodo.mx' actualizó precio de Conector RJ45 de $4.50 a $5.00 por inflación de proveedor.</t>
+  </si>
+  <si>
+    <t>LOG-CPV-03</t>
+  </si>
+  <si>
+    <t>Baja / Devolución</t>
+  </si>
+  <si>
+    <t>Al registrar devolución a proveedor, mercancía defectuosa o baja</t>
+  </si>
+  <si>
+    <t>id_producto, id_user, categoria='compraventa', accion='Baja / Devolución', comentario, documentacion</t>
+  </si>
+  <si>
+    <t>Descuenta piezas del inventario vendible y genera folio de salida para reclamo de garantía.</t>
+  </si>
+  <si>
+    <t>Nota de crédito, guía de paquetería de devolución o reporte de garantía.</t>
+  </si>
+  <si>
+    <t>[Devolución] Usuario 'carlos.almacen' registró devolución a proveedor de 10 Switches 8 puertos defectuosos.</t>
+  </si>
+  <si>
+    <t>LOG-VEH-01</t>
+  </si>
+  <si>
+    <t>Vehículos</t>
+  </si>
+  <si>
+    <t>Al guardar nuevo vehículo en módulo de flotilla</t>
+  </si>
+  <si>
+    <t>id_producto, id_user, categoria='vehiculos', accion='Alta de vehículo', comentario, documentacion</t>
+  </si>
+  <si>
+    <t>Registra unidad con número de serie VIN, placas, año, modelo y responsable asignado en flotilla.</t>
+  </si>
+  <si>
+    <t>Tarjeta de circulación, factura vehicular, póliza de seguro y fotografías 360°.</t>
+  </si>
+  <si>
+    <t>[Alta] Usuario 'admin@nodo.mx' registró Nissan NP300 2023, Placas: XX-1234-A, Asignado a: Logística.</t>
+  </si>
+  <si>
+    <t>LOG-VEH-02</t>
+  </si>
+  <si>
+    <t>Edición / Reasignación</t>
+  </si>
+  <si>
+    <t>Al modificar datos de la unidad o cambiar chofer responsable</t>
+  </si>
+  <si>
+    <t>id_producto, id_user, categoria='vehiculos', accion='Actualización / Reasignación', comentario</t>
+  </si>
+  <si>
+    <t>Actualiza el custodio 'A cargo de quién está' que se muestra en el Dashboard de Mantenimientos.</t>
+  </si>
+  <si>
+    <t>Carta responsiva vehicular firmada con checklist de entrega-recepción.</t>
+  </si>
+  <si>
+    <t>[Reasignación] Usuario 'admin@nodo.mx' asignó unidad Hilux (Placas: YY-9876) a cargo de 'Roberto Gómez'.</t>
+  </si>
+  <si>
+    <t>LOG-VEH-03</t>
+  </si>
+  <si>
+    <t>Mantenimiento</t>
+  </si>
+  <si>
+    <t>Al registrar servicio de afinación, llantas, frenos o reparación</t>
+  </si>
+  <si>
+    <t>id_producto, id_user, categoria='vehiculos', accion='Registro de mantenimiento', comentario, documentacion</t>
+  </si>
+  <si>
+    <t>Calcula próximo servicio, actualiza kilometraje actual y suma al costo acumulado del vehículo.</t>
+  </si>
+  <si>
+    <t>Factura fiscal del taller mecánico, orden de servicio y bitácora de mantenimiento.</t>
+  </si>
+  <si>
+    <t>[Mantenimiento] Usuario 'almacen@nodo.mx' registró afinación a 45,000 km. Costo: $4,200. Taller: AutoExpress.</t>
+  </si>
+  <si>
+    <t>LOG-VEH-04</t>
+  </si>
+  <si>
+    <t>Baja de Unidad</t>
+  </si>
+  <si>
+    <t>Al desincorporar vehículo por venta, siniestro total o fin de vida útil</t>
+  </si>
+  <si>
+    <t>id_producto, id_user, categoria='vehiculos', accion='Baja de unidad vehicular', comentario (motivo), acta</t>
+  </si>
+  <si>
+    <t>Pasa a estatus inactivo; cancela alertas de mantenimiento pendientes y desvincula al chofer.</t>
+  </si>
+  <si>
+    <t>Factura de venta, finiquito de aseguradora o baja vehicular de placas ante secretaría.</t>
+  </si>
+  <si>
+    <t>[Baja] Usuario 'superadmin@nodo.mx' dio de baja Chevrolet Spark por pérdida total dictaminada por seguro.</t>
+  </si>
+  <si>
+    <t>LOG-USR-01</t>
+  </si>
+  <si>
+    <t>Alta / Edición de Usuario</t>
+  </si>
+  <si>
+    <t>Usuarios y Roles</t>
+  </si>
+  <si>
+    <t>Al crear o modificar usuarios, restablecer contraseñas o asignar roles</t>
+  </si>
+  <si>
+    <t>id_user, id_rol, categoria='sistema', accion='Alta / Modificación de usuario', comentario</t>
+  </si>
+  <si>
+    <t>Otorga o revoca privilegios en la aplicación de acuerdo con la jerarquía definida.</t>
+  </si>
+  <si>
+    <t>Solicitud de alta de usuario por Recursos Humanos o jefatura de departamento.</t>
+  </si>
+  <si>
+    <t>[Usuarios] Super Admin asignó el rol 'Almacenistas' al usuario 'luis.perez@nodo.mx'.</t>
+  </si>
+  <si>
+    <t>Crítica</t>
+  </si>
+  <si>
+    <t>ESPECIFICACIÓN TÉCNICA DE LA TABLA DE LOGS (`movimientos`)</t>
+  </si>
+  <si>
+    <t>Columna / Campo</t>
+  </si>
+  <si>
+    <t>Tipo de Dato MySQL</t>
+  </si>
+  <si>
+    <t>Nulo / Default</t>
+  </si>
+  <si>
+    <t>Clave / Índice</t>
+  </si>
+  <si>
+    <t>Descripción Técnica y Propósito</t>
+  </si>
+  <si>
+    <t>Regla de Negocio / Restricción</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>BIGINT UNSIGNED</t>
+  </si>
+  <si>
+    <t>NO / AUTO_INCREMENT</t>
+  </si>
+  <si>
+    <t>PRIMARY KEY</t>
+  </si>
+  <si>
+    <t>Identificador secuencial único de la entrada de log.</t>
+  </si>
+  <si>
+    <t>Autogenerado e inmutable.</t>
+  </si>
+  <si>
+    <t>id_user</t>
+  </si>
+  <si>
+    <t>INT UNSIGNED</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>INDEX</t>
+  </si>
+  <si>
+    <t>ID del usuario autenticado que ejecutó la operación.</t>
+  </si>
+  <si>
+    <t>Debe existir en la tabla `users`.</t>
+  </si>
+  <si>
+    <t>id_producto</t>
+  </si>
+  <si>
+    <t>YES (NULL)</t>
+  </si>
+  <si>
+    <t>ID del activo, consumible, producto de venta o vehículo afectado.</t>
+  </si>
+  <si>
+    <t>NULL si la acción es general del sistema.</t>
+  </si>
+  <si>
+    <t>categoria</t>
+  </si>
+  <si>
+    <t>VARCHAR(50)</t>
+  </si>
+  <si>
+    <t>Módulo origen ('fijos', 'consumibles', 'compraventa', 'vehiculos', 'sistema').</t>
+  </si>
+  <si>
+    <t>Permite filtros rápidos por módulo.</t>
+  </si>
+  <si>
+    <t>accion</t>
+  </si>
+  <si>
+    <t>VARCHAR(150)</t>
+  </si>
+  <si>
+    <t>Nombre descriptivo de la acción ('Alta', 'Consumo', 'Baja', 'Edición').</t>
+  </si>
+  <si>
+    <t>Estandarizado para reportes y métricas.</t>
+  </si>
+  <si>
+    <t>comentario</t>
+  </si>
+  <si>
+    <t>TEXT</t>
+  </si>
+  <si>
+    <t>NONE</t>
+  </si>
+  <si>
+    <t>Detalle explicativo, motivo del consumo, cantidades o campos modificados.</t>
+  </si>
+  <si>
+    <t>Obligatorio en Bajas y Consumos.</t>
+  </si>
+  <si>
+    <t>documentacion</t>
+  </si>
+  <si>
+    <t>VARCHAR(255)</t>
+  </si>
+  <si>
+    <t>Ruta relativa del archivo adjunto (acta, factura, remisión, foto).</t>
+  </si>
+  <si>
+    <t>Almacenado en storage/uploads/.</t>
+  </si>
+  <si>
+    <t>created_at</t>
+  </si>
+  <si>
+    <t>TIMESTAMP</t>
+  </si>
+  <si>
+    <t>NO / CURRENT_TIMESTAMP</t>
+  </si>
+  <si>
+    <t>Fecha y hora exacta en que ocurrió la operación en el servidor.</t>
+  </si>
+  <si>
+    <t>No modificable; orden cronológico.</t>
+  </si>
+  <si>
+    <t>updated_at</t>
+  </si>
+  <si>
+    <t>YES / NULL</t>
+  </si>
+  <si>
+    <t>Timestamp de control Eloquent.</t>
+  </si>
+  <si>
+    <t>Auditoría interna.</t>
+  </si>
+  <si>
+    <t>POLÍTICAS DE SEGURIDAD, INTEGRIDAD Y GOBERNANZA DE AUDITORÍA</t>
+  </si>
+  <si>
+    <t>1. INMUTABILIDAD TOTAL: Las filas de auditoría no pueden ser alteradas ni eliminadas bajo ninguna circunstancia, ni siquiera por el rol Super Admin.</t>
+  </si>
+  <si>
+    <t>2. NO REPUDIO: Cada registro almacena el identificador único del usuario que realizó la acción (`id_user`), garantizando responsabilidad individual.</t>
+  </si>
+  <si>
+    <t>3. JUSTIFICACIÓN OBLIGATORIA: En operaciones de 'Baja' y 'Consumo de Insumos', el sistema exige un comentario descriptivo y, en caso de bajas, documento sustentatorio.</t>
+  </si>
+  <si>
+    <t>4. MONITOREO DE STOCK: El consumo de consumibles actualiza el saldo de inmediato; si el inventario llega a ≤ 10%, el sistema activa las alertas en el Dashboard y la campana de notificaciones.</t>
+  </si>
+  <si>
+    <t>5. EXPORTABILIDAD: Esta especificación garantiza que los registros pueden auditarse y exportarse a hojas de cálculo para revisiones de control interno y contraloría.</t>
   </si>
 </sst>
 </file>
@@ -526,7 +1114,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="21">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -617,8 +1205,107 @@
       <color rgb="FF991B1B"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b val="0"/>
+      <i val="1"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF475569"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="12"/>
+      <color rgb="FF1E3A8A"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="8.5"/>
+      <color rgb="FF1E293B"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="9"/>
+      <color rgb="FF10B981"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="9"/>
+      <color rgb="FFF59E0B"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="9"/>
+      <color rgb="FFEF4444"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="9"/>
+      <color rgb="FFB91C1C"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="9"/>
+      <color rgb="FF1E3A8A"/>
+      <name val="Consolas"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="9.5"/>
+      <color rgb="FF0F172A"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -643,8 +1330,62 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF10B981"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1F5F9"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3B82F6"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEF4444"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF59E0B"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6366F1"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF334155"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -667,11 +1408,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF0F172A"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF0F172A"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF0F172A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF0F172A"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="40">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
@@ -708,6 +1464,79 @@
     </xf>
     <xf xfId="0" fontId="9" numFmtId="0" fillId="4" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="10" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="11" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="12" numFmtId="0" fillId="5" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="13" numFmtId="0" fillId="6" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="12" numFmtId="0" fillId="7" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="12" numFmtId="0" fillId="8" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="12" numFmtId="0" fillId="9" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="12" numFmtId="0" fillId="10" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="12" numFmtId="0" fillId="2" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="14" numFmtId="0" fillId="11" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="14" numFmtId="0" fillId="11" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="15" numFmtId="0" fillId="11" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="14" numFmtId="0" fillId="12" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="14" numFmtId="0" fillId="12" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="16" numFmtId="0" fillId="12" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="17" numFmtId="0" fillId="11" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="15" numFmtId="0" fillId="12" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="16" numFmtId="0" fillId="11" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="17" numFmtId="0" fillId="12" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="18" numFmtId="0" fillId="11" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="12" numFmtId="0" fillId="13" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="19" numFmtId="0" fillId="11" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="19" numFmtId="0" fillId="12" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="20" numFmtId="0" fillId="12" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1011,12 +1840,12 @@
   <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="29.279" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="24.565" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="29.279" customWidth="true" style="0"/>
+    <col min="2" max="2" width="16.425" customWidth="true" style="0"/>
+    <col min="3" max="3" width="10.426" customWidth="true" style="0"/>
+    <col min="4" max="4" width="12.854" customWidth="true" style="0"/>
+    <col min="5" max="5" width="22.28" customWidth="true" style="0"/>
+    <col min="6" max="6" width="24.565" customWidth="true" style="0"/>
     <col min="7" max="7" width="60" customWidth="true" style="0"/>
   </cols>
   <sheetData>
@@ -1179,14 +2008,14 @@
   <dimension ref="A1:H128"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="6.998" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="57.7" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="19.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="43.561" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="25.851" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="24.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="22.28" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="6.998" customWidth="true" style="0"/>
+    <col min="2" max="2" width="57.7" customWidth="true" style="0"/>
+    <col min="3" max="3" width="19.995" customWidth="true" style="0"/>
+    <col min="4" max="4" width="43.561" customWidth="true" style="0"/>
+    <col min="5" max="5" width="23.423" customWidth="true" style="0"/>
+    <col min="6" max="6" width="25.851" customWidth="true" style="0"/>
+    <col min="7" max="7" width="24.708" customWidth="true" style="0"/>
+    <col min="8" max="8" width="22.28" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -4468,4 +5297,930 @@
   </headerFooter>
   <tableParts count="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:J48"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="true" style="0"/>
+    <col min="2" max="2" width="18" customWidth="true" style="0"/>
+    <col min="3" max="3" width="16" customWidth="true" style="0"/>
+    <col min="4" max="4" width="26" customWidth="true" style="0"/>
+    <col min="5" max="5" width="30" customWidth="true" style="0"/>
+    <col min="6" max="6" width="30" customWidth="true" style="0"/>
+    <col min="7" max="7" width="26" customWidth="true" style="0"/>
+    <col min="8" max="8" width="22" customWidth="true" style="0"/>
+    <col min="9" max="9" width="38" customWidth="true" style="0"/>
+    <col min="10" max="10" width="14" customWidth="true" style="0"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="15" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="16" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="16" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="17" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="B6" s="18"/>
+      <c r="C6" s="20" t="s">
+        <v>173</v>
+      </c>
+      <c r="D6" s="20"/>
+      <c r="E6" s="21" t="s">
+        <v>175</v>
+      </c>
+      <c r="F6" s="21"/>
+      <c r="G6" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="H6" s="22"/>
+      <c r="I6" s="23" t="s">
+        <v>179</v>
+      </c>
+      <c r="J6" s="23"/>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="B7" s="19"/>
+      <c r="C7" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="J7" s="19"/>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="19"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="17" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" customHeight="1" ht="28">
+      <c r="A12" s="24" t="s">
+        <v>182</v>
+      </c>
+      <c r="B12" s="24" t="s">
+        <v>183</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>184</v>
+      </c>
+      <c r="D12" s="24" t="s">
+        <v>185</v>
+      </c>
+      <c r="E12" s="24" t="s">
+        <v>186</v>
+      </c>
+      <c r="F12" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="G12" s="24" t="s">
+        <v>188</v>
+      </c>
+      <c r="H12" s="24" t="s">
+        <v>189</v>
+      </c>
+      <c r="I12" s="24" t="s">
+        <v>190</v>
+      </c>
+      <c r="J12" s="24" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" customHeight="1" ht="40">
+      <c r="A13" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="B13" s="26" t="s">
+        <v>193</v>
+      </c>
+      <c r="C13" s="26" t="s">
+        <v>194</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>195</v>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>196</v>
+      </c>
+      <c r="F13" s="25" t="s">
+        <v>197</v>
+      </c>
+      <c r="G13" s="25" t="s">
+        <v>198</v>
+      </c>
+      <c r="H13" s="25" t="s">
+        <v>199</v>
+      </c>
+      <c r="I13" s="25" t="s">
+        <v>200</v>
+      </c>
+      <c r="J13" s="27" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" customHeight="1" ht="40">
+      <c r="A14" s="29" t="s">
+        <v>202</v>
+      </c>
+      <c r="B14" s="29" t="s">
+        <v>203</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>194</v>
+      </c>
+      <c r="D14" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="E14" s="28" t="s">
+        <v>205</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>206</v>
+      </c>
+      <c r="G14" s="28" t="s">
+        <v>207</v>
+      </c>
+      <c r="H14" s="28" t="s">
+        <v>208</v>
+      </c>
+      <c r="I14" s="28" t="s">
+        <v>209</v>
+      </c>
+      <c r="J14" s="30" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" customHeight="1" ht="40">
+      <c r="A15" s="26" t="s">
+        <v>211</v>
+      </c>
+      <c r="B15" s="26" t="s">
+        <v>212</v>
+      </c>
+      <c r="C15" s="26" t="s">
+        <v>194</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>213</v>
+      </c>
+      <c r="E15" s="25" t="s">
+        <v>214</v>
+      </c>
+      <c r="F15" s="25" t="s">
+        <v>215</v>
+      </c>
+      <c r="G15" s="25" t="s">
+        <v>216</v>
+      </c>
+      <c r="H15" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="I15" s="25" t="s">
+        <v>217</v>
+      </c>
+      <c r="J15" s="31" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" customHeight="1" ht="40">
+      <c r="A16" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="B16" s="29" t="s">
+        <v>193</v>
+      </c>
+      <c r="C16" s="29" t="s">
+        <v>220</v>
+      </c>
+      <c r="D16" s="28" t="s">
+        <v>221</v>
+      </c>
+      <c r="E16" s="28" t="s">
+        <v>222</v>
+      </c>
+      <c r="F16" s="28" t="s">
+        <v>223</v>
+      </c>
+      <c r="G16" s="28" t="s">
+        <v>224</v>
+      </c>
+      <c r="H16" s="28" t="s">
+        <v>199</v>
+      </c>
+      <c r="I16" s="28" t="s">
+        <v>225</v>
+      </c>
+      <c r="J16" s="32" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" customHeight="1" ht="40">
+      <c r="A17" s="26" t="s">
+        <v>226</v>
+      </c>
+      <c r="B17" s="26" t="s">
+        <v>227</v>
+      </c>
+      <c r="C17" s="26" t="s">
+        <v>220</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>228</v>
+      </c>
+      <c r="E17" s="25" t="s">
+        <v>229</v>
+      </c>
+      <c r="F17" s="25" t="s">
+        <v>230</v>
+      </c>
+      <c r="G17" s="25" t="s">
+        <v>231</v>
+      </c>
+      <c r="H17" s="25" t="s">
+        <v>232</v>
+      </c>
+      <c r="I17" s="25" t="s">
+        <v>233</v>
+      </c>
+      <c r="J17" s="33" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" customHeight="1" ht="40">
+      <c r="A18" s="29" t="s">
+        <v>234</v>
+      </c>
+      <c r="B18" s="29" t="s">
+        <v>235</v>
+      </c>
+      <c r="C18" s="29" t="s">
+        <v>220</v>
+      </c>
+      <c r="D18" s="28" t="s">
+        <v>236</v>
+      </c>
+      <c r="E18" s="28" t="s">
+        <v>237</v>
+      </c>
+      <c r="F18" s="28" t="s">
+        <v>238</v>
+      </c>
+      <c r="G18" s="28" t="s">
+        <v>239</v>
+      </c>
+      <c r="H18" s="28" t="s">
+        <v>199</v>
+      </c>
+      <c r="I18" s="28" t="s">
+        <v>240</v>
+      </c>
+      <c r="J18" s="32" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" customHeight="1" ht="40">
+      <c r="A19" s="26" t="s">
+        <v>241</v>
+      </c>
+      <c r="B19" s="26" t="s">
+        <v>242</v>
+      </c>
+      <c r="C19" s="26" t="s">
+        <v>220</v>
+      </c>
+      <c r="D19" s="25" t="s">
+        <v>243</v>
+      </c>
+      <c r="E19" s="25" t="s">
+        <v>244</v>
+      </c>
+      <c r="F19" s="25" t="s">
+        <v>245</v>
+      </c>
+      <c r="G19" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="H19" s="25" t="s">
+        <v>208</v>
+      </c>
+      <c r="I19" s="25" t="s">
+        <v>247</v>
+      </c>
+      <c r="J19" s="31" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" customHeight="1" ht="40">
+      <c r="A20" s="29" t="s">
+        <v>248</v>
+      </c>
+      <c r="B20" s="29" t="s">
+        <v>193</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>249</v>
+      </c>
+      <c r="D20" s="28" t="s">
+        <v>250</v>
+      </c>
+      <c r="E20" s="28" t="s">
+        <v>251</v>
+      </c>
+      <c r="F20" s="28" t="s">
+        <v>252</v>
+      </c>
+      <c r="G20" s="28" t="s">
+        <v>253</v>
+      </c>
+      <c r="H20" s="28" t="s">
+        <v>199</v>
+      </c>
+      <c r="I20" s="28" t="s">
+        <v>254</v>
+      </c>
+      <c r="J20" s="32" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" customHeight="1" ht="40">
+      <c r="A21" s="26" t="s">
+        <v>255</v>
+      </c>
+      <c r="B21" s="26" t="s">
+        <v>256</v>
+      </c>
+      <c r="C21" s="26" t="s">
+        <v>249</v>
+      </c>
+      <c r="D21" s="25" t="s">
+        <v>257</v>
+      </c>
+      <c r="E21" s="25" t="s">
+        <v>258</v>
+      </c>
+      <c r="F21" s="25" t="s">
+        <v>259</v>
+      </c>
+      <c r="G21" s="25" t="s">
+        <v>260</v>
+      </c>
+      <c r="H21" s="25" t="s">
+        <v>208</v>
+      </c>
+      <c r="I21" s="25" t="s">
+        <v>261</v>
+      </c>
+      <c r="J21" s="33" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" customHeight="1" ht="40">
+      <c r="A22" s="29" t="s">
+        <v>262</v>
+      </c>
+      <c r="B22" s="29" t="s">
+        <v>263</v>
+      </c>
+      <c r="C22" s="29" t="s">
+        <v>249</v>
+      </c>
+      <c r="D22" s="28" t="s">
+        <v>264</v>
+      </c>
+      <c r="E22" s="28" t="s">
+        <v>265</v>
+      </c>
+      <c r="F22" s="28" t="s">
+        <v>266</v>
+      </c>
+      <c r="G22" s="28" t="s">
+        <v>267</v>
+      </c>
+      <c r="H22" s="28" t="s">
+        <v>208</v>
+      </c>
+      <c r="I22" s="28" t="s">
+        <v>268</v>
+      </c>
+      <c r="J22" s="34" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" customHeight="1" ht="40">
+      <c r="A23" s="26" t="s">
+        <v>269</v>
+      </c>
+      <c r="B23" s="26" t="s">
+        <v>193</v>
+      </c>
+      <c r="C23" s="26" t="s">
+        <v>270</v>
+      </c>
+      <c r="D23" s="25" t="s">
+        <v>271</v>
+      </c>
+      <c r="E23" s="25" t="s">
+        <v>272</v>
+      </c>
+      <c r="F23" s="25" t="s">
+        <v>273</v>
+      </c>
+      <c r="G23" s="25" t="s">
+        <v>274</v>
+      </c>
+      <c r="H23" s="25" t="s">
+        <v>208</v>
+      </c>
+      <c r="I23" s="25" t="s">
+        <v>275</v>
+      </c>
+      <c r="J23" s="27" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" customHeight="1" ht="40">
+      <c r="A24" s="29" t="s">
+        <v>276</v>
+      </c>
+      <c r="B24" s="29" t="s">
+        <v>277</v>
+      </c>
+      <c r="C24" s="29" t="s">
+        <v>270</v>
+      </c>
+      <c r="D24" s="28" t="s">
+        <v>278</v>
+      </c>
+      <c r="E24" s="28" t="s">
+        <v>279</v>
+      </c>
+      <c r="F24" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G24" s="28" t="s">
+        <v>281</v>
+      </c>
+      <c r="H24" s="28" t="s">
+        <v>208</v>
+      </c>
+      <c r="I24" s="28" t="s">
+        <v>282</v>
+      </c>
+      <c r="J24" s="30" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" customHeight="1" ht="40">
+      <c r="A25" s="26" t="s">
+        <v>283</v>
+      </c>
+      <c r="B25" s="26" t="s">
+        <v>284</v>
+      </c>
+      <c r="C25" s="26" t="s">
+        <v>270</v>
+      </c>
+      <c r="D25" s="25" t="s">
+        <v>285</v>
+      </c>
+      <c r="E25" s="25" t="s">
+        <v>286</v>
+      </c>
+      <c r="F25" s="25" t="s">
+        <v>287</v>
+      </c>
+      <c r="G25" s="25" t="s">
+        <v>288</v>
+      </c>
+      <c r="H25" s="25" t="s">
+        <v>199</v>
+      </c>
+      <c r="I25" s="25" t="s">
+        <v>289</v>
+      </c>
+      <c r="J25" s="27" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" customHeight="1" ht="40">
+      <c r="A26" s="29" t="s">
+        <v>290</v>
+      </c>
+      <c r="B26" s="29" t="s">
+        <v>291</v>
+      </c>
+      <c r="C26" s="29" t="s">
+        <v>270</v>
+      </c>
+      <c r="D26" s="28" t="s">
+        <v>292</v>
+      </c>
+      <c r="E26" s="28" t="s">
+        <v>293</v>
+      </c>
+      <c r="F26" s="28" t="s">
+        <v>294</v>
+      </c>
+      <c r="G26" s="28" t="s">
+        <v>295</v>
+      </c>
+      <c r="H26" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="I26" s="28" t="s">
+        <v>296</v>
+      </c>
+      <c r="J26" s="34" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" customHeight="1" ht="40">
+      <c r="A27" s="26" t="s">
+        <v>297</v>
+      </c>
+      <c r="B27" s="26" t="s">
+        <v>298</v>
+      </c>
+      <c r="C27" s="26" t="s">
+        <v>299</v>
+      </c>
+      <c r="D27" s="25" t="s">
+        <v>300</v>
+      </c>
+      <c r="E27" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="F27" s="25" t="s">
+        <v>302</v>
+      </c>
+      <c r="G27" s="25" t="s">
+        <v>303</v>
+      </c>
+      <c r="H27" s="25" t="s">
+        <v>208</v>
+      </c>
+      <c r="I27" s="25" t="s">
+        <v>304</v>
+      </c>
+      <c r="J27" s="35" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10">
+      <c r="A30" s="17" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" customHeight="1" ht="24">
+      <c r="A31" s="36" t="s">
+        <v>307</v>
+      </c>
+      <c r="B31" s="36" t="s">
+        <v>308</v>
+      </c>
+      <c r="C31" s="36" t="s">
+        <v>309</v>
+      </c>
+      <c r="D31" s="36" t="s">
+        <v>310</v>
+      </c>
+      <c r="E31" s="36" t="s">
+        <v>311</v>
+      </c>
+      <c r="F31" s="36" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" customHeight="1" ht="22">
+      <c r="A32" s="37" t="s">
+        <v>313</v>
+      </c>
+      <c r="B32" s="26" t="s">
+        <v>314</v>
+      </c>
+      <c r="C32" s="26" t="s">
+        <v>315</v>
+      </c>
+      <c r="D32" s="26" t="s">
+        <v>316</v>
+      </c>
+      <c r="E32" s="25" t="s">
+        <v>317</v>
+      </c>
+      <c r="F32" s="25" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" customHeight="1" ht="22">
+      <c r="A33" s="38" t="s">
+        <v>319</v>
+      </c>
+      <c r="B33" s="29" t="s">
+        <v>320</v>
+      </c>
+      <c r="C33" s="29" t="s">
+        <v>321</v>
+      </c>
+      <c r="D33" s="29" t="s">
+        <v>322</v>
+      </c>
+      <c r="E33" s="28" t="s">
+        <v>323</v>
+      </c>
+      <c r="F33" s="28" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" customHeight="1" ht="22">
+      <c r="A34" s="37" t="s">
+        <v>325</v>
+      </c>
+      <c r="B34" s="26" t="s">
+        <v>320</v>
+      </c>
+      <c r="C34" s="26" t="s">
+        <v>326</v>
+      </c>
+      <c r="D34" s="26" t="s">
+        <v>322</v>
+      </c>
+      <c r="E34" s="25" t="s">
+        <v>327</v>
+      </c>
+      <c r="F34" s="25" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" customHeight="1" ht="22">
+      <c r="A35" s="38" t="s">
+        <v>329</v>
+      </c>
+      <c r="B35" s="29" t="s">
+        <v>330</v>
+      </c>
+      <c r="C35" s="29" t="s">
+        <v>321</v>
+      </c>
+      <c r="D35" s="29" t="s">
+        <v>322</v>
+      </c>
+      <c r="E35" s="28" t="s">
+        <v>331</v>
+      </c>
+      <c r="F35" s="28" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" customHeight="1" ht="22">
+      <c r="A36" s="37" t="s">
+        <v>333</v>
+      </c>
+      <c r="B36" s="26" t="s">
+        <v>334</v>
+      </c>
+      <c r="C36" s="26" t="s">
+        <v>321</v>
+      </c>
+      <c r="D36" s="26" t="s">
+        <v>322</v>
+      </c>
+      <c r="E36" s="25" t="s">
+        <v>335</v>
+      </c>
+      <c r="F36" s="25" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" customHeight="1" ht="22">
+      <c r="A37" s="38" t="s">
+        <v>337</v>
+      </c>
+      <c r="B37" s="29" t="s">
+        <v>338</v>
+      </c>
+      <c r="C37" s="29" t="s">
+        <v>326</v>
+      </c>
+      <c r="D37" s="29" t="s">
+        <v>339</v>
+      </c>
+      <c r="E37" s="28" t="s">
+        <v>340</v>
+      </c>
+      <c r="F37" s="28" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" customHeight="1" ht="22">
+      <c r="A38" s="37" t="s">
+        <v>342</v>
+      </c>
+      <c r="B38" s="26" t="s">
+        <v>343</v>
+      </c>
+      <c r="C38" s="26" t="s">
+        <v>326</v>
+      </c>
+      <c r="D38" s="26" t="s">
+        <v>339</v>
+      </c>
+      <c r="E38" s="25" t="s">
+        <v>344</v>
+      </c>
+      <c r="F38" s="25" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" customHeight="1" ht="22">
+      <c r="A39" s="38" t="s">
+        <v>346</v>
+      </c>
+      <c r="B39" s="29" t="s">
+        <v>347</v>
+      </c>
+      <c r="C39" s="29" t="s">
+        <v>348</v>
+      </c>
+      <c r="D39" s="29" t="s">
+        <v>322</v>
+      </c>
+      <c r="E39" s="28" t="s">
+        <v>349</v>
+      </c>
+      <c r="F39" s="28" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" customHeight="1" ht="22">
+      <c r="A40" s="37" t="s">
+        <v>351</v>
+      </c>
+      <c r="B40" s="26" t="s">
+        <v>347</v>
+      </c>
+      <c r="C40" s="26" t="s">
+        <v>352</v>
+      </c>
+      <c r="D40" s="26" t="s">
+        <v>339</v>
+      </c>
+      <c r="E40" s="25" t="s">
+        <v>353</v>
+      </c>
+      <c r="F40" s="25" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10">
+      <c r="A43" s="17" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" customHeight="1" ht="22">
+      <c r="A44" s="39" t="s">
+        <v>356</v>
+      </c>
+      <c r="B44" s="39"/>
+      <c r="C44" s="39"/>
+      <c r="D44" s="39"/>
+      <c r="E44" s="39"/>
+      <c r="F44" s="39"/>
+      <c r="G44" s="39"/>
+      <c r="H44" s="39"/>
+      <c r="I44" s="39"/>
+      <c r="J44" s="39"/>
+    </row>
+    <row r="45" spans="1:10" customHeight="1" ht="22">
+      <c r="A45" s="39" t="s">
+        <v>357</v>
+      </c>
+      <c r="B45" s="39"/>
+      <c r="C45" s="39"/>
+      <c r="D45" s="39"/>
+      <c r="E45" s="39"/>
+      <c r="F45" s="39"/>
+      <c r="G45" s="39"/>
+      <c r="H45" s="39"/>
+      <c r="I45" s="39"/>
+      <c r="J45" s="39"/>
+    </row>
+    <row r="46" spans="1:10" customHeight="1" ht="22">
+      <c r="A46" s="39" t="s">
+        <v>358</v>
+      </c>
+      <c r="B46" s="39"/>
+      <c r="C46" s="39"/>
+      <c r="D46" s="39"/>
+      <c r="E46" s="39"/>
+      <c r="F46" s="39"/>
+      <c r="G46" s="39"/>
+      <c r="H46" s="39"/>
+      <c r="I46" s="39"/>
+      <c r="J46" s="39"/>
+    </row>
+    <row r="47" spans="1:10" customHeight="1" ht="22">
+      <c r="A47" s="39" t="s">
+        <v>359</v>
+      </c>
+      <c r="B47" s="39"/>
+      <c r="C47" s="39"/>
+      <c r="D47" s="39"/>
+      <c r="E47" s="39"/>
+      <c r="F47" s="39"/>
+      <c r="G47" s="39"/>
+      <c r="H47" s="39"/>
+      <c r="I47" s="39"/>
+      <c r="J47" s="39"/>
+    </row>
+    <row r="48" spans="1:10" customHeight="1" ht="22">
+      <c r="A48" s="39" t="s">
+        <v>360</v>
+      </c>
+      <c r="B48" s="39"/>
+      <c r="C48" s="39"/>
+      <c r="D48" s="39"/>
+      <c r="E48" s="39"/>
+      <c r="F48" s="39"/>
+      <c r="G48" s="39"/>
+      <c r="H48" s="39"/>
+      <c r="I48" s="39"/>
+      <c r="J48" s="39"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B8"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D8"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E7:F8"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H8"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="I7:J8"/>
+    <mergeCell ref="A44:J44"/>
+    <mergeCell ref="A45:J45"/>
+    <mergeCell ref="A46:J46"/>
+    <mergeCell ref="A47:J47"/>
+    <mergeCell ref="A48:J48"/>
+  </mergeCells>
+  <printOptions gridLines="false" gridLinesSet="true"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="0"/>
+</worksheet>
 </file>
</xml_diff>